<commit_message>
#9 #8 Order Placement Completed.
</commit_message>
<xml_diff>
--- a/Design-Files/Knob-PCB-v1.0/Deliverables/BOM/Client_BOM_Knob-PCB-v1.0.xlsx
+++ b/Design-Files/Knob-PCB-v1.0/Deliverables/BOM/Client_BOM_Knob-PCB-v1.0.xlsx
@@ -5,7 +5,7 @@
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="153222"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark-consultants\dustinm-lampleddriver\Design-Files\Knob-PCB-v1.0\Deliverables\BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark-Consultants\dustinm-lampleddriver\Design-Files\Knob-PCB-v1.0\Deliverables\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="115">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="165" uniqueCount="120">
   <si>
     <t>#</t>
   </si>
@@ -364,6 +364,22 @@
   </si>
   <si>
     <t>Do Not Place</t>
+  </si>
+  <si>
+    <t>Peripheral</t>
+  </si>
+  <si>
+    <t>Antenna</t>
+  </si>
+  <si>
+    <t>high gain embedded 2.4g Wifi U.FL Ble FPC Flexible Antenna ufl internal Antenna flexible Ble BT Antenna for ESP32 Module</t>
+  </si>
+  <si>
+    <t>ZXWIFI24I408</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Signal Plus
+</t>
   </si>
 </sst>
 </file>
@@ -581,9 +597,6 @@
     <xf numFmtId="0" fontId="5" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -592,6 +605,9 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -880,22 +896,22 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:K23"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:K24"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="3.109375" style="4" customWidth="1"/>
-    <col min="3" max="3" width="18.6640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="3.140625" style="4" customWidth="1"/>
+    <col min="3" max="3" width="18.7109375" style="4" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="36" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="30" customWidth="1"/>
-    <col min="6" max="6" width="26.5546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="33.44140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="21.44140625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="17.88671875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="16.6640625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="29.44140625" customWidth="1"/>
+    <col min="6" max="6" width="26.5703125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="33.42578125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="21.42578125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="17.85546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="16.7109375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="29.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1"/>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
@@ -904,11 +920,11 @@
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
       <c r="H1" s="2"/>
-      <c r="I1" s="14"/>
-      <c r="J1" s="14"/>
-      <c r="K1" s="14"/>
-    </row>
-    <row r="2" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="I1" s="17"/>
+      <c r="J1" s="17"/>
+      <c r="K1" s="17"/>
+    </row>
+    <row r="2" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
       <c r="B2" s="5" t="s">
         <v>0</v>
@@ -941,7 +957,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="48.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:11" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1"/>
       <c r="B3" s="11">
         <f>ROW(B3) - ROW($B$2)</f>
@@ -973,7 +989,7 @@
       </c>
       <c r="K3" s="7"/>
     </row>
-    <row r="4" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1"/>
       <c r="B4" s="11">
         <f t="shared" ref="B4:B22" si="0">ROW(B4) - ROW($B$2)</f>
@@ -1005,7 +1021,7 @@
       </c>
       <c r="K4" s="9"/>
     </row>
-    <row r="5" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1"/>
       <c r="B5" s="11">
         <f>ROW(B5) - ROW($B$2)</f>
@@ -1037,7 +1053,7 @@
       </c>
       <c r="K5" s="7"/>
     </row>
-    <row r="6" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="1"/>
       <c r="B6" s="11">
         <f t="shared" si="0"/>
@@ -1069,7 +1085,7 @@
       </c>
       <c r="K6" s="9"/>
     </row>
-    <row r="7" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="1"/>
       <c r="B7" s="11">
         <f>ROW(B7) - ROW($B$2)</f>
@@ -1101,7 +1117,7 @@
       </c>
       <c r="K7" s="7"/>
     </row>
-    <row r="8" spans="1:11" ht="36.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
       <c r="B8" s="11">
         <f t="shared" si="0"/>
@@ -1133,7 +1149,7 @@
       </c>
       <c r="K8" s="9"/>
     </row>
-    <row r="9" spans="1:11" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
       <c r="B9" s="11">
         <f>ROW(B9) - ROW($B$2)</f>
@@ -1165,7 +1181,7 @@
       </c>
       <c r="K9" s="7"/>
     </row>
-    <row r="10" spans="1:11" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:11" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="1"/>
       <c r="B10" s="11">
         <f t="shared" si="0"/>
@@ -1197,7 +1213,7 @@
       </c>
       <c r="K10" s="9"/>
     </row>
-    <row r="11" spans="1:11" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:11" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="1"/>
       <c r="B11" s="11">
         <f>ROW(B11) - ROW($B$2)</f>
@@ -1229,7 +1245,7 @@
       </c>
       <c r="K11" s="7"/>
     </row>
-    <row r="12" spans="1:11" ht="48.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:11" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="1"/>
       <c r="B12" s="11">
         <f t="shared" si="0"/>
@@ -1261,7 +1277,7 @@
       </c>
       <c r="K12" s="9"/>
     </row>
-    <row r="13" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="1"/>
       <c r="B13" s="11">
         <f>ROW(B13) - ROW($B$2)</f>
@@ -1293,7 +1309,7 @@
       </c>
       <c r="K13" s="7"/>
     </row>
-    <row r="14" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="1"/>
       <c r="B14" s="11">
         <f t="shared" si="0"/>
@@ -1325,7 +1341,7 @@
       </c>
       <c r="K14" s="9"/>
     </row>
-    <row r="15" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="1"/>
       <c r="B15" s="11">
         <f>ROW(B15) - ROW($B$2)</f>
@@ -1357,47 +1373,49 @@
       </c>
       <c r="K15" s="7"/>
     </row>
-    <row r="16" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="1"/>
       <c r="B16" s="11">
         <f t="shared" si="0"/>
         <v>14</v>
       </c>
-      <c r="C16" s="17" t="s">
+      <c r="C16" s="16" t="s">
         <v>8</v>
       </c>
-      <c r="D16" s="16" t="s">
+      <c r="D16" s="15" t="s">
         <v>27</v>
       </c>
-      <c r="E16" s="15" t="s">
+      <c r="E16" s="14" t="s">
         <v>46</v>
       </c>
-      <c r="F16" s="16" t="s">
+      <c r="F16" s="15" t="s">
         <v>63</v>
       </c>
-      <c r="G16" s="15" t="s">
+      <c r="G16" s="14" t="s">
         <v>79</v>
       </c>
-      <c r="H16" s="16" t="s">
+      <c r="H16" s="15" t="s">
         <v>94</v>
       </c>
-      <c r="I16" s="15" t="s">
+      <c r="I16" s="14" t="s">
         <v>107</v>
       </c>
-      <c r="J16" s="16">
+      <c r="J16" s="15">
         <v>3</v>
       </c>
-      <c r="K16" s="16" t="s">
+      <c r="K16" s="15" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="17" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="1"/>
       <c r="B17" s="11">
         <f>ROW(B17) - ROW($B$2)</f>
         <v>15</v>
       </c>
-      <c r="C17" s="12"/>
+      <c r="C17" s="13" t="s">
+        <v>8</v>
+      </c>
       <c r="D17" s="7" t="s">
         <v>28</v>
       </c>
@@ -1421,7 +1439,7 @@
       </c>
       <c r="K17" s="7"/>
     </row>
-    <row r="18" spans="1:11" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="1"/>
       <c r="B18" s="11">
         <f t="shared" si="0"/>
@@ -1453,7 +1471,7 @@
       </c>
       <c r="K18" s="9"/>
     </row>
-    <row r="19" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="1"/>
       <c r="B19" s="11">
         <f>ROW(B19) - ROW($B$2)</f>
@@ -1485,7 +1503,7 @@
       </c>
       <c r="K19" s="7"/>
     </row>
-    <row r="20" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="1"/>
       <c r="B20" s="11">
         <f t="shared" si="0"/>
@@ -1517,7 +1535,7 @@
       </c>
       <c r="K20" s="9"/>
     </row>
-    <row r="21" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="1"/>
       <c r="B21" s="11">
         <f>ROW(B21) - ROW($B$2)</f>
@@ -1549,7 +1567,7 @@
       </c>
       <c r="K21" s="7"/>
     </row>
-    <row r="22" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="1"/>
       <c r="B22" s="11">
         <f t="shared" si="0"/>
@@ -1581,7 +1599,7 @@
       </c>
       <c r="K22" s="9"/>
     </row>
-    <row r="23" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="1"/>
       <c r="B23" s="11">
         <f>ROW(B23) - ROW($B$2)</f>
@@ -1612,6 +1630,37 @@
         <v>1</v>
       </c>
       <c r="K23" s="7"/>
+    </row>
+    <row r="24" spans="1:11" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B24" s="11">
+        <f>ROW(B24) - ROW($B$2)</f>
+        <v>22</v>
+      </c>
+      <c r="C24" s="12" t="s">
+        <v>115</v>
+      </c>
+      <c r="D24" s="7" t="s">
+        <v>116</v>
+      </c>
+      <c r="E24" s="8" t="s">
+        <v>117</v>
+      </c>
+      <c r="F24" s="7" t="s">
+        <v>113</v>
+      </c>
+      <c r="G24" s="8" t="s">
+        <v>118</v>
+      </c>
+      <c r="H24" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="I24" s="8" t="s">
+        <v>112</v>
+      </c>
+      <c r="J24" s="7">
+        <v>1</v>
+      </c>
+      <c r="K24" s="7"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
#8 Motor Peripheral added in Knob BOM
</commit_message>
<xml_diff>
--- a/Design-Files/Knob-PCB-v1.0/Deliverables/BOM/Client_BOM_Knob-PCB-v1.0.xlsx
+++ b/Design-Files/Knob-PCB-v1.0/Deliverables/BOM/Client_BOM_Knob-PCB-v1.0.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="165" uniqueCount="120">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="124">
   <si>
     <t>#</t>
   </si>
@@ -380,6 +380,18 @@
   <si>
     <t xml:space="preserve">Signal Plus
 </t>
+  </si>
+  <si>
+    <t>Three Phase Brushless Gimbal Stabilizer Motor</t>
+  </si>
+  <si>
+    <t>Motor</t>
+  </si>
+  <si>
+    <t>EM3215 3-Phase Brushless DC Motor</t>
+  </si>
+  <si>
+    <t>SparkFun</t>
   </si>
 </sst>
 </file>
@@ -896,7 +908,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:K24"/>
+  <dimension ref="A1:K25"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="3.140625" style="4" customWidth="1"/>
@@ -1662,6 +1674,37 @@
       </c>
       <c r="K24" s="7"/>
     </row>
+    <row r="25" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B25" s="11">
+        <f>ROW(B25) - ROW($B$2)</f>
+        <v>23</v>
+      </c>
+      <c r="C25" s="12" t="s">
+        <v>115</v>
+      </c>
+      <c r="D25" s="7" t="s">
+        <v>121</v>
+      </c>
+      <c r="E25" s="8" t="s">
+        <v>120</v>
+      </c>
+      <c r="F25" s="7" t="s">
+        <v>113</v>
+      </c>
+      <c r="G25" s="8" t="s">
+        <v>122</v>
+      </c>
+      <c r="H25" s="7" t="s">
+        <v>123</v>
+      </c>
+      <c r="I25" s="8" t="s">
+        <v>112</v>
+      </c>
+      <c r="J25" s="7">
+        <v>1</v>
+      </c>
+      <c r="K25" s="7"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="I1:K1"/>

</xml_diff>